<commit_message>
Add race and life rhythm systems
</commit_message>
<xml_diff>
--- a/assets_cropped/Sirius Symboli/manifest_edit.xlsx
+++ b/assets_cropped/Sirius Symboli/manifest_edit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\TanukiProject\tanuki_app\assets_cropped\Sirius Symboli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007F64AB-1CFA-473C-957B-E22BDA3E42DB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81224E2A-F3D5-4C39-A355-A46AF567A549}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="139">
   <si>
     <t>filename</t>
   </si>
@@ -68,9 +68,6 @@
     <t>idle_mix_dance_me-smile.gif</t>
   </si>
   <si>
-    <t>shared_food_request</t>
-  </si>
-  <si>
     <t>idle_mix_dance-smile.gif</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>low,severe</t>
   </si>
   <si>
-    <t>window_perch,offer_timeout_route_a_step2,random</t>
-  </si>
-  <si>
     <t>idle_side-cool.gif</t>
   </si>
   <si>
@@ -125,314 +119,357 @@
     <t>idle_side-sad.gif</t>
   </si>
   <si>
-    <t>window_perch,care_companion,relation_watch,honey_guard_take,random</t>
-  </si>
-  <si>
     <t>idle_side-scold.gif</t>
   </si>
   <si>
+    <t>idle_side-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_talk-sad.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_talk-shock.gif</t>
+  </si>
+  <si>
+    <t>idle_sit_talk-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_sit-happy.gif</t>
+  </si>
+  <si>
+    <t>window_perch,care_companion,relation_close,bottle_feed_watch,random</t>
+  </si>
+  <si>
+    <t>idle_sit-sad.gif</t>
+  </si>
+  <si>
+    <t>window_perch,care_companion,relation_close,honey_guard_take,bottle_feed_watch,random</t>
+  </si>
+  <si>
+    <t>idle_sit-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_stand_hand-cool.gif</t>
+  </si>
+  <si>
+    <t>idle_stand_hand-glance.gif</t>
+  </si>
+  <si>
+    <t>idle_stand_hand-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_stand_hand-sad.gif</t>
+  </si>
+  <si>
+    <t>offer_preview,offer_timeout_route_a_step1,shared_food_hold,shared_food_watch</t>
+  </si>
+  <si>
+    <t>idle_stand_hand-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_stand_tail-cool.gif</t>
+  </si>
+  <si>
+    <t>post_observe</t>
+  </si>
+  <si>
+    <t>idle_stand_tail-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_stand_tail-smile.gif</t>
+  </si>
+  <si>
+    <t>idle_stand-angry.gif</t>
+  </si>
+  <si>
+    <t>idle_stand-cool.gif</t>
+  </si>
+  <si>
+    <t>idle_stand-happy.gif</t>
+  </si>
+  <si>
+    <t>idle_stand-sad.gif</t>
+  </si>
+  <si>
+    <t>window_perch,honey_guard_take,shared_food_react,random</t>
+  </si>
+  <si>
+    <t>idle_stand-smile.gif</t>
+  </si>
+  <si>
+    <t>interaction_idle_drink_Teio-happy.gif</t>
+  </si>
+  <si>
+    <t>interaction,care_interaction,care_interaction_teio</t>
+  </si>
+  <si>
+    <t>interaction_idle_rub_face_Tsuyoshi-happy.gif</t>
+  </si>
+  <si>
+    <t>interaction,care_interaction,care_interaction_tsuyoshi</t>
+  </si>
+  <si>
+    <t>interaction_idle_tail_Teio-happy.gif</t>
+  </si>
+  <si>
+    <t>move_fly-smile.gif</t>
+  </si>
+  <si>
+    <t>window_flight</t>
+  </si>
+  <si>
+    <t>move_jog-happy.gif</t>
+  </si>
+  <si>
+    <t>move_run_hand_drink-smile.gif</t>
+  </si>
+  <si>
+    <t>future_work,care_approach_teio</t>
+  </si>
+  <si>
+    <t>move_run_hand-angry.gif</t>
+  </si>
+  <si>
+    <t>honey_guard_move</t>
+  </si>
+  <si>
+    <t>move_run_hand-happy.gif</t>
+  </si>
+  <si>
+    <t>move_run_hand-scold.gif</t>
+  </si>
+  <si>
+    <t>honey_guard_move,negative_reaction</t>
+  </si>
+  <si>
+    <t>move_run-angry.gif</t>
+  </si>
+  <si>
+    <t>move_run-cool.gif</t>
+  </si>
+  <si>
+    <t>move_run-happy.gif</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>move_run-sad.gif</t>
+  </si>
+  <si>
+    <t>move_run-scold.gif</t>
+  </si>
+  <si>
+    <t>negative_reaction</t>
+  </si>
+  <si>
+    <t>move_run-smile.gif</t>
+  </si>
+  <si>
+    <t>move_walk_drink-happy.gif</t>
+  </si>
+  <si>
+    <t>offer_accept_honey</t>
+  </si>
+  <si>
+    <t>move_walk_talk-happy.gif</t>
+  </si>
+  <si>
+    <t>move_walk_talk-sad.gif</t>
+  </si>
+  <si>
+    <t>move_walk_talk-scold.gif</t>
+  </si>
+  <si>
+    <t>move_walk-angry.gif</t>
+  </si>
+  <si>
+    <t>move_walk-happy.gif</t>
+  </si>
+  <si>
+    <t>move_walk-sad.gif</t>
+  </si>
+  <si>
+    <t>window_walk,random</t>
+  </si>
+  <si>
+    <t>move_walk-smile.gif</t>
+  </si>
+  <si>
+    <t>backup_original_filename</t>
+  </si>
+  <si>
+    <t>backup_character</t>
+  </si>
+  <si>
+    <t>backup_reason</t>
+  </si>
+  <si>
+    <t>darg_original_sad.gif__Sirius Symboli</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>darg_original_sad.gif</t>
+  </si>
+  <si>
+    <t>Sirius Symboli</t>
+  </si>
+  <si>
+    <t>stale_filename_not_found</t>
+  </si>
+  <si>
+    <t>idle_sing-smile.gif__Sirius Symboli</t>
+  </si>
+  <si>
+    <t>idle_sing-smile.gif</t>
+  </si>
+  <si>
+    <t>offer_accept_honey,shared_food_consume</t>
+  </si>
+  <si>
+    <t>offer_timeout_route_b_step1,shared_food_watch,shared_food_hold</t>
+  </si>
+  <si>
+    <t>offer_preview,shared_food_hold,shared_food_watch</t>
+  </si>
+  <si>
+    <t>window_walk,random,shared_food_approach</t>
+  </si>
+  <si>
+    <t>idle_rest-angry.gif</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>idle_rest-angry-sleep.gif</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>idle_rest-sleep.gif</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>idle_rest-smile.gif</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>low,severe</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>normal</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>activity_sleeping</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>activity_sleep_settling,activity_sleep_waking</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>random,activity_sleep_join_approach</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>idle_rest-cool.gif</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>activity_sleep_join_settling</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>random</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,random,shared_food_approach,activity_race_to_start</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_walk,offer_timeout_route_a_step3,random,activity_sleep_join_approach,activity_race_to_start</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>honey_guard_move,activity_race_running</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>random,activity_race_running</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>random,shared_food_approach,activity_race_running_teio</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>care_approach</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>care_companion,observe_hold,bottle_feed_watch,activity_sleep_observing,activity_race_finish_win</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_companion,relation_watch,honey_guard_take,random,activity_race_finish_lose</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
     <t>offer_timeout_route_b_step2,negative_reaction</t>
-  </si>
-  <si>
-    <t>idle_side-smile.gif</t>
-  </si>
-  <si>
-    <t>window_perch,care_companion,relation_close,random</t>
-  </si>
-  <si>
-    <t>idle_sit_talk-sad.gif</t>
-  </si>
-  <si>
-    <t>care_companion,observe_hold,honey_guard_take,shared_food_react</t>
-  </si>
-  <si>
-    <t>idle_sit_talk-shock.gif</t>
-  </si>
-  <si>
-    <t>idle_sit_talk-smile.gif</t>
-  </si>
-  <si>
-    <t>care_companion,observe_hold,shared_food_react</t>
-  </si>
-  <si>
-    <t>idle_sit-happy.gif</t>
-  </si>
-  <si>
-    <t>window_perch,care_companion,relation_close,bottle_feed_watch,random</t>
-  </si>
-  <si>
-    <t>idle_sit-sad.gif</t>
-  </si>
-  <si>
-    <t>window_perch,care_companion,relation_close,honey_guard_take,bottle_feed_watch,random</t>
-  </si>
-  <si>
-    <t>idle_sit-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_stand_hand-cool.gif</t>
-  </si>
-  <si>
-    <t>idle_stand_hand-glance.gif</t>
-  </si>
-  <si>
-    <t>idle_stand_hand-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_stand_hand-sad.gif</t>
-  </si>
-  <si>
-    <t>offer_preview,offer_timeout_route_a_step1,shared_food_hold,shared_food_watch</t>
-  </si>
-  <si>
-    <t>idle_stand_hand-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_stand_tail-cool.gif</t>
-  </si>
-  <si>
-    <t>post_observe</t>
-  </si>
-  <si>
-    <t>idle_stand_tail-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_stand_tail-smile.gif</t>
-  </si>
-  <si>
-    <t>idle_stand-angry.gif</t>
-  </si>
-  <si>
-    <t>window_perch,post_observe,random</t>
-  </si>
-  <si>
-    <t>idle_stand-cool.gif</t>
-  </si>
-  <si>
-    <t>bottle_feed_watch,shared_food_react</t>
-  </si>
-  <si>
-    <t>idle_stand-happy.gif</t>
-  </si>
-  <si>
-    <t>idle_stand-sad.gif</t>
-  </si>
-  <si>
-    <t>window_perch,honey_guard_take,shared_food_react,random</t>
-  </si>
-  <si>
-    <t>idle_stand-smile.gif</t>
-  </si>
-  <si>
-    <t>interaction_idle_drink_Teio-happy.gif</t>
-  </si>
-  <si>
-    <t>interaction,care_interaction,care_interaction_teio</t>
-  </si>
-  <si>
-    <t>interaction_idle_rub_face_Tsuyoshi-happy.gif</t>
-  </si>
-  <si>
-    <t>interaction,care_interaction,care_interaction_tsuyoshi</t>
-  </si>
-  <si>
-    <t>interaction_idle_tail_Teio-happy.gif</t>
-  </si>
-  <si>
-    <t>move_fly-smile.gif</t>
-  </si>
-  <si>
-    <t>window_flight</t>
-  </si>
-  <si>
-    <t>move_jog-happy.gif</t>
-  </si>
-  <si>
-    <t>move_run_hand_drink-smile.gif</t>
-  </si>
-  <si>
-    <t>future_work,care_approach_teio</t>
-  </si>
-  <si>
-    <t>move_run_hand-angry.gif</t>
-  </si>
-  <si>
-    <t>honey_guard_move</t>
-  </si>
-  <si>
-    <t>move_run_hand-happy.gif</t>
-  </si>
-  <si>
-    <t>move_run_hand-scold.gif</t>
-  </si>
-  <si>
-    <t>honey_guard_move,negative_reaction</t>
-  </si>
-  <si>
-    <t>move_run-angry.gif</t>
-  </si>
-  <si>
-    <t>move_run-cool.gif</t>
-  </si>
-  <si>
-    <t>future_work,care_approach</t>
-  </si>
-  <si>
-    <t>move_run-happy.gif</t>
-  </si>
-  <si>
-    <t>random</t>
-  </si>
-  <si>
-    <t>move_run-sad.gif</t>
-  </si>
-  <si>
-    <t>move_run-scold.gif</t>
-  </si>
-  <si>
-    <t>negative_reaction</t>
-  </si>
-  <si>
-    <t>move_run-smile.gif</t>
-  </si>
-  <si>
-    <t>move_walk_drink-happy.gif</t>
-  </si>
-  <si>
-    <t>offer_accept_honey</t>
-  </si>
-  <si>
-    <t>move_walk_talk-happy.gif</t>
-  </si>
-  <si>
-    <t>move_walk_talk-sad.gif</t>
-  </si>
-  <si>
-    <t>move_walk_talk-scold.gif</t>
-  </si>
-  <si>
-    <t>move_walk-angry.gif</t>
-  </si>
-  <si>
-    <t>move_walk-happy.gif</t>
-  </si>
-  <si>
-    <t>move_walk-sad.gif</t>
-  </si>
-  <si>
-    <t>window_walk,random</t>
-  </si>
-  <si>
-    <t>move_walk-smile.gif</t>
-  </si>
-  <si>
-    <t>backup_original_filename</t>
-  </si>
-  <si>
-    <t>backup_character</t>
-  </si>
-  <si>
-    <t>backup_reason</t>
-  </si>
-  <si>
-    <t>darg_original_sad.gif__Sirius Symboli</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>darg_original_sad.gif</t>
-  </si>
-  <si>
-    <t>Sirius Symboli</t>
-  </si>
-  <si>
-    <t>stale_filename_not_found</t>
-  </si>
-  <si>
-    <t>idle_sing-smile.gif__Sirius Symboli</t>
-  </si>
-  <si>
-    <t>idle_sing-smile.gif</t>
-  </si>
-  <si>
-    <t>offer_accept_honey,shared_food_consume</t>
-  </si>
-  <si>
-    <t>bottle_feed_hold,shared_food_watch,shared_food_hold</t>
-  </si>
-  <si>
-    <t>offer_timeout_route_b_step1,shared_food_watch,shared_food_hold</t>
-  </si>
-  <si>
-    <t>offer_preview,shared_food_hold,shared_food_watch</t>
-  </si>
-  <si>
-    <t>window_perch,random,shared_food_react</t>
-  </si>
-  <si>
-    <t>random,shared_food_approach</t>
-  </si>
-  <si>
-    <t>window_walk,random,shared_food_approach</t>
-  </si>
-  <si>
-    <t>idle_rest-angry.gif</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>idle_rest-angry-sleep.gif</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>idle_rest-sleep.gif</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>idle_rest-smile.gif</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>low,severe</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>normal</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>activity_sleeping</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>activity_sleep_settling,activity_sleep_waking</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>care_companion,observe_hold,bottle_feed_watch,activity_sleep_observing</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>random,activity_sleep_join_approach</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>idle_rest-cool.gif</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>activity_sleep_join_settling</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>random</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>window_walk,offer_timeout_route_a_step3,random,activity_sleep_join_approach</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,offer_timeout_route_a_step2,random,activity_race_ready,activity_race_finish_lose</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>post_observe,activity_race_finish_win</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>care_companion,observe_hold,shared_food_react,activity_race_recovery</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>care_companion,observe_hold,honey_guard_take,shared_food_react,activity_race_recovery</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>shared_food_request,activity_race_challenge</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>bottle_feed_watch,shared_food_react,activity_race_accept</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>bottle_feed_hold,shared_food_watch,shared_food_hold,activity_race_accept</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,random,shared_food_react,activity_race_decline</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>random,activity_race_running_teio</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,care_companion,relation_close,random,activity_race_ready,activity_race_finish_lose</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,random,shared_food_react,activity_race_consider</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>window_perch,post_observe,random,activity_race_decline,activity_race_consider</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -788,7 +825,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -843,8 +880,8 @@
       <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
+      <c r="C7" s="2" t="s">
+        <v>131</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -852,13 +889,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
         <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -866,13 +903,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
         <v>18</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -880,13 +917,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -894,13 +931,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -908,13 +945,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -922,13 +959,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -936,13 +973,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -950,13 +987,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -964,13 +1001,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -978,13 +1015,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -992,13 +1029,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1006,13 +1043,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1020,13 +1057,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1034,13 +1071,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
         <v>26</v>
       </c>
-      <c r="B21" t="s">
-        <v>27</v>
-      </c>
-      <c r="C21" t="s">
-        <v>28</v>
+      <c r="C21" s="2" t="s">
+        <v>127</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1048,13 +1085,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
         <v>6</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1062,13 +1099,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
         <v>30</v>
-      </c>
-      <c r="B23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" t="s">
-        <v>32</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1076,13 +1113,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" t="s">
-        <v>34</v>
+        <v>26</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>125</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1090,13 +1127,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
         <v>6</v>
       </c>
-      <c r="C25" t="s">
-        <v>36</v>
+      <c r="C25" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1104,13 +1141,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" t="s">
-        <v>38</v>
+        <v>29</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1118,13 +1155,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C27" t="s">
-        <v>40</v>
+        <v>26</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>130</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1132,13 +1169,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
         <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1146,13 +1183,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
-      </c>
-      <c r="C29" t="s">
-        <v>43</v>
+        <v>29</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>129</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1160,13 +1197,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1174,13 +1211,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C31" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1188,13 +1225,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C32" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -1202,13 +1239,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B33" t="s">
         <v>6</v>
       </c>
-      <c r="C33" t="s">
-        <v>113</v>
+      <c r="C33" s="2" t="s">
+        <v>133</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -1216,13 +1253,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B34" t="s">
         <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -1230,13 +1267,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C35" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -1244,13 +1281,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C36" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -1258,13 +1295,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C37" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1272,13 +1309,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B38" t="s">
         <v>6</v>
       </c>
-      <c r="C38" t="s">
-        <v>56</v>
+      <c r="C38" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1286,13 +1323,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B39" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C39" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1300,13 +1337,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B40" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C40" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1314,13 +1351,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B41" t="s">
-        <v>27</v>
-      </c>
-      <c r="C41" t="s">
-        <v>60</v>
+        <v>26</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>138</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1328,13 +1365,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B42" t="s">
         <v>6</v>
       </c>
-      <c r="C42" t="s">
-        <v>62</v>
+      <c r="C42" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1342,13 +1379,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B43" t="s">
-        <v>31</v>
-      </c>
-      <c r="C43" t="s">
-        <v>116</v>
+        <v>29</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -1356,13 +1393,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="B44" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C44" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1370,13 +1407,13 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B45" t="s">
-        <v>31</v>
-      </c>
-      <c r="C45" t="s">
-        <v>116</v>
+        <v>29</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>137</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -1384,13 +1421,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
         <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -1401,13 +1438,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B47" t="s">
         <v>6</v>
       </c>
       <c r="C47" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -1418,13 +1455,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B48" t="s">
         <v>6</v>
       </c>
       <c r="C48" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -1435,13 +1472,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B49" t="s">
         <v>6</v>
       </c>
       <c r="C49" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -1449,13 +1486,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="B50" t="s">
-        <v>31</v>
-      </c>
-      <c r="C50" t="s">
-        <v>117</v>
+        <v>29</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -1463,13 +1500,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B51" t="s">
         <v>6</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -1477,13 +1514,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B52" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C52" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -1491,13 +1528,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="B53" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C53" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -1505,13 +1542,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="B54" t="s">
         <v>6</v>
       </c>
       <c r="C54" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -1519,13 +1556,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B55" t="s">
-        <v>27</v>
-      </c>
-      <c r="C55" t="s">
-        <v>78</v>
+        <v>26</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>120</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -1533,13 +1570,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B56" t="s">
         <v>6</v>
       </c>
-      <c r="C56" t="s">
-        <v>84</v>
+      <c r="C56" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -1547,13 +1584,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B57" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C57" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -1561,13 +1598,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B58" t="s">
-        <v>27</v>
-      </c>
-      <c r="C58" t="s">
-        <v>86</v>
+        <v>26</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>135</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -1575,13 +1612,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B59" t="s">
         <v>6</v>
       </c>
       <c r="C59" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D59">
         <v>1</v>
@@ -1589,13 +1626,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B60" t="s">
-        <v>31</v>
-      </c>
-      <c r="C60" t="s">
-        <v>86</v>
+        <v>29</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="D60">
         <v>1</v>
@@ -1603,13 +1640,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B61" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C61" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -1617,13 +1654,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B62" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -1631,13 +1668,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B63" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="D63">
         <v>1</v>
@@ -1645,13 +1682,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B64" t="s">
         <v>6</v>
       </c>
       <c r="C64" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D64">
         <v>1</v>
@@ -1659,13 +1696,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B65" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="D65">
         <v>1</v>
@@ -1673,13 +1710,13 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B66" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C66" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D66">
         <v>1</v>
@@ -1687,13 +1724,13 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B67" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C67" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D67">
         <v>1</v>
@@ -1701,12 +1738,12 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B68" t="s">
-        <v>31</v>
-      </c>
-      <c r="C68" t="s">
+        <v>29</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>118</v>
       </c>
       <c r="D68">
@@ -1742,18 +1779,18 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="G1" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="H1" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -1762,45 +1799,45 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="F2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="H2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="F3" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="G3" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="H3" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>